<commit_message>
added mother data set with salaries
</commit_message>
<xml_diff>
--- a/data/wage_per_country.xlsx
+++ b/data/wage_per_country.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michelenaorourke/Desktop/6.C51/1.C51/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michelenaorourke/Desktop/6.C51/1.C51/1.C51-Final-Project/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CF08285D-EBC1-C74C-88F2-C9FE829DB832}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACA470D8-DA44-3846-AC3E-E2DE7C82D865}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="900" windowWidth="28040" windowHeight="17180" xr2:uid="{E2C66FE1-D308-9F49-86F4-0EC69F38E64D}"/>
+    <workbookView xWindow="1080" yWindow="860" windowWidth="28040" windowHeight="17180" xr2:uid="{E2C66FE1-D308-9F49-86F4-0EC69F38E64D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -41,9 +41,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
-    <t>US</t>
-  </si>
-  <si>
     <t>Spain</t>
   </si>
   <si>
@@ -59,9 +56,6 @@
     <t>Mexico</t>
   </si>
   <si>
-    <t>Russia</t>
-  </si>
-  <si>
     <t>Portugal</t>
   </si>
   <si>
@@ -183,6 +177,12 @@
   </si>
   <si>
     <t>Country</t>
+  </si>
+  <si>
+    <t>United States of America</t>
+  </si>
+  <si>
+    <t>Russian Federation</t>
   </si>
 </sst>
 </file>
@@ -579,15 +579,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="B2" s="1">
         <v>55819</v>
@@ -595,7 +595,7 @@
     </row>
     <row r="3" spans="1:2" ht="20" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B3" s="2">
         <v>37500</v>
@@ -603,7 +603,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B4">
         <v>4509.6000000000004</v>
@@ -611,7 +611,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B5" s="3">
         <v>12877.81</v>
@@ -619,7 +619,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6" s="3">
         <v>26240.14</v>
@@ -627,7 +627,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" s="3">
         <v>9018.86</v>
@@ -635,7 +635,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="B8" s="3">
         <v>11616.07</v>
@@ -643,7 +643,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B9" s="3">
         <v>26705.79</v>
@@ -651,7 +651,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B10" s="3">
         <v>5808</v>
@@ -659,7 +659,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B11" s="3">
         <v>14122</v>
@@ -667,7 +667,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B12" s="3">
         <v>11963.92</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B13" s="3">
         <v>10531.43</v>
@@ -683,7 +683,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B14" s="3">
         <v>19604.88</v>
@@ -691,7 +691,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B15" s="3">
         <v>56861.95</v>
@@ -699,7 +699,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B16" s="3">
         <v>12285.78</v>
@@ -707,7 +707,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B17" s="3">
         <v>16266.82</v>
@@ -715,7 +715,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B18" s="3">
         <v>6596.52</v>
@@ -723,7 +723,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B19" s="4">
         <v>43833.79</v>
@@ -731,7 +731,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B20" s="3">
         <v>6655.62</v>
@@ -739,7 +739,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B21" s="3">
         <v>4278.24</v>
@@ -747,7 +747,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B22" s="3">
         <v>2051.1</v>
@@ -755,7 +755,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B23" s="3">
         <v>11196.48</v>
@@ -763,7 +763,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B24" s="3">
         <v>9190.58</v>
@@ -771,7 +771,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B25" s="3">
         <v>4514.3999999999996</v>
@@ -779,7 +779,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B26" s="3">
         <v>848.28</v>
@@ -787,7 +787,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B27" s="3">
         <v>5979.99</v>
@@ -795,7 +795,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B28" s="3">
         <v>13027.27</v>
@@ -803,7 +803,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B29" s="3">
         <v>2424</v>
@@ -811,7 +811,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B30" s="3">
         <v>6395.79</v>
@@ -819,7 +819,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B31" s="3">
         <v>11888.72</v>
@@ -827,7 +827,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B32" s="3">
         <v>51635.89</v>
@@ -835,7 +835,7 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B33" s="3">
         <v>1533</v>
@@ -843,7 +843,7 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B34" s="3">
         <v>24382.55</v>
@@ -851,7 +851,7 @@
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B35" s="3">
         <v>40902.1</v>
@@ -859,7 +859,7 @@
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B36" s="3">
         <v>3324.12</v>
@@ -867,7 +867,7 @@
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B37" s="3">
         <v>4800</v>
@@ -875,7 +875,7 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B38" s="3">
         <v>13891.95</v>
@@ -883,7 +883,7 @@
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B39" s="3">
         <v>12196.79</v>
@@ -891,7 +891,7 @@
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B40" s="1">
         <v>8170</v>
@@ -899,7 +899,7 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B41" s="3">
         <v>1276</v>
@@ -907,7 +907,7 @@
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B42" s="3">
         <v>9805.56</v>
@@ -915,7 +915,7 @@
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B43" s="3">
         <v>10042.56</v>
@@ -923,7 +923,7 @@
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B44" s="3">
         <v>6677.28</v>
@@ -931,7 +931,7 @@
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B45" s="3">
         <v>2007.5</v>
@@ -939,7 +939,7 @@
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B46" s="3">
         <v>2811.72</v>
@@ -947,7 +947,7 @@
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B47" s="3">
         <v>45400.44</v>

</xml_diff>